<commit_message>
Workbook: anchor detail sheets on hand-built YAML rank, not universe rank.
After the 2026-07-01 refresh promoted 118 new PROXY candidates, the
universe-wide top-30 filled with PROXY names and pushed the hand-built
REAL YAMLs (TKA, GTCO, 6305, etc.) below rank 30 — so the detail-sheet
selector (which scanned universe_rr[:30] for source==REAL) only emitted
3 detail sheets (LOCAL, LAC, SZG).

Fix: select the top-10 detail sheets from the candidates list directly,
which load_candidates() already sorts by each YAML's own bottom-up
reward/risk ratio. Detail sheets are now stable regardless of how many
PROXY candidates flood the universe ranking.

Restored to 10 detail sheets: LOCAL, LAC, SZG, TKA, ELUX-B, GTCO,
6305, DSI, 241560, ETL.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVNbiVw8xFVKcK527PvUF9
</commit_message>
<xml_diff>
--- a/output/cyclepapa_risk_reward_workbook.xlsx
+++ b/output/cyclepapa_risk_reward_workbook.xlsx
@@ -18,7 +18,14 @@
     <sheet name="LOCAL" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="LAC" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="SZG" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Methodology" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="TKA" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ELUX-B" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="GTCO" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="6305" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DSI" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="241560" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="ETL" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Methodology" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -601,7 +608,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Generated 2026-07-01</t>
+          <t>Generated 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -2208,6 +2215,4587 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Thyssenkrupp AG (Steel Europe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TKA  ·  DE  ·  Bucket A  ·  Archetype A1, A2, H  ·  Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.34×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.55× / 2.30× / 4.20×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>7.1×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>3.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>EU_industrial_policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2024-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>A1 + A2 + H — Daniel Kretinsky's EPCG took 20pct stake in Thyssenkrupp Steel Europe subsidiary July 2024 (€1.0-1.5bn implied valuation). JV with German State pending (Lower Saxony + federal govt). €2bn EU state aid for green-steel transition approved Jul 2023 (SA.103861). Multi-decade decarbonisation pivot: Hydrogen-DRI plant Salzgitter site; Marine Systems carve-out worth €1-1.5bn separately. Iduna Aurelius industrial JV pending under EU IAA framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Thyssenkrupp Steel JV with German state closes (Kretinsky 50pct / state 50pct)</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-09-30</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.6-2.4× / Down -0.2--0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Marine Systems carve-out / IPO completion</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.4-1.8× / Down -0.05--0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>European steel cycle inflection (HRC &gt;€600/t)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2028-06-30</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.5-2.2× / Down -0.2--0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>SALCOS first green-steel production at converted Duisburg blast furnace</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.3-1.8× / Down -0.15--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: 0.4x book with €2bn approved state aid + Marine
+Systems €1-1.5bn carve-out implies SOTP gap to ~€4-5bn vs
+current cap €3.2bn.
+Leg 2: Kretinsky 20pct in Steel sub + Krupp-Stiftung 21pct
+in parent = aligned cap-stack.
+Leg 3: PARTIAL — Kretinsky stake = revealed preference;
+KfW second-tranche commit not yet placed; Carlyle Marine
+interest is signal but not signed.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>EPCG / Daniel Kretinsky, German Federal State + Lower Saxony, Krupp-Stiftung foundation (21pct legacy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="n"/>
+      <c r="C41" s="19" t="n"/>
+      <c r="D41" s="19" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="n"/>
+      <c r="C45" s="19" t="n"/>
+      <c r="D45" s="19" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Kretinsky / state JV terms materially worsen (state share &lt;40pct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>SALCOS Phase 1 slips beyond mid-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>CBAM materially watered down by EU Council</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Marine Systems carve-out cancelled or distressed sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="n"/>
+      <c r="C51" s="19" t="n"/>
+      <c r="D51" s="19" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr"/>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is end-2027 and TKA is down 60pct from current ~€5.
+Most likely: Steel-JV negotiations stalled on state commitment;
+Marine Systems carve-out priced at distressed multiple; SALCOS
+cost overran by €1bn; Chinese steel dumping intensified; multiple
+to 0.3x book; another asset disposal at distressed terms.
+Second most likely: EU IAA fiscal envelope cut in EU budget
+negotiation; KfW declined; SALCOS deferred.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="inlineStr"/>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype A1 (Kretinsky 20pct + Krupp-Stiftung 21pct
+aligned anchors) + A2 (EU state aid €2bn) + H (governance reset
+via Steel-JV restructure). Universe score 0.95 = 7th-highest;
+multi-leg catalyst structure puts it in Tier 1 (4 dated catalysts
++ 2 floors).
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="38">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AB Electrolux (Series B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ELUX-B  ·  SE  ·  Bucket A  ·  Archetype A1, D  ·  Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.32×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.55× / 2.20× / 4.00×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>6.7×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.9×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Nordic_consumer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>multiple_norm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>SEK 9,062m fully underwritten rights issue (subscription Jun 2-16, 2026); Investor AB (Wallenberg) subscribes pro-rata SEK 1.7bn + guarantees additional SEK 1.7bn = 37.56% of issue. Tied to strategic partnership with Midea for North America, global organization optimization, and footprint restructuring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D2 Issue Discount Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D3 Backstop Cost Pct</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D5 Delta Wam Months</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>D6 Debt Tranches Post</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>D7 Ucc Terminations Pm30D</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>D8 Mip Strike Over Recap</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>D9B Anchor Premium To Recap</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>D9C Premium To Vwap</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>D9D Liquidation Recovery Pct</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>D13 Altman Z</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>Midea North America partnership operational ramp</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.6-2.5× / Down -0.2--0.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>Global organization &amp; footprint optimization completion</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2027-06-30</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.4-2.0× / Down -0.15--0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Appliance cycle (US housing + EU disinflation) bottom</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2027-06-30</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.5-2.2× / Down -0.15--0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: Appliance multiples compressed; Whirlpool/peers trade at
+distressed margins; Electrolux's mid-cycle EBITDA on its
+pre-collapse base implies material upside on multiple
+normalisation alone.
+Leg 2: Investor AB (Wallenberg) as backstop is the cleanest
+natural-owner Nordic anchor pattern; Midea as strategic JV
+partner is Archetype D customer-aligned anchor; fully
+underwritten = no rump risk; EGM passed May 27 = governance
+settled.
+Leg 3: Investor AB undertaking 37.56% of the issue (pro-rata
++ guarantee) is the revealed-preference signal. They could
+have taken just pro-rata; the additional SEK 1.7bn guarantee
+on market terms is the asymmetric commitment.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="n"/>
+      <c r="C46" s="19" t="n"/>
+      <c r="D46" s="19" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Investor AB (Wallenberg Foundations), Midea Group (strategic JV partner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>17.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Midea JV terminated or delayed beyond H1 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>US administration imposes punitive tariffs on China-affiliated JVs that void North America economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Investor AB sells beyond pro-rata commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Cost-out programme misses Q2 FY27 milestone by &gt;25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Second equity raise needed within 18 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="n"/>
+      <c r="C61" s="19" t="n"/>
+      <c r="D61" s="19" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="20" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is end-2027 and ELUX-B is down 70% from rights price.
+Most likely cause: Midea JV economics undermined by US-China
+trade frictions (tariff escalation, FDI screening, executive
+order action against Chinese ownership in North American
+consumer appliance market). Wallenberg held its position but
+growth thesis evaporated; legacy European appliance market
+did not recover as expected.
+Second-most-likely cause: Cost-out programme execution failed
+(factory transitions slipped; severance costs ballooned; one-off
+impairments cascaded). Q3 FY27 print missed materially; analyst
+downgrades cascaded.
+Where this would show up first: US executive-order activity on
+Chinese appliance JVs; quarterly factory-transition milestones
+in interim reports; Midea quarterly disclosures.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B64" s="19" t="n"/>
+      <c r="C64" s="19" t="n"/>
+      <c r="D64" s="19" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype A1 (Wallenberg as long-term natural-owner
+anchor at pro-rata + guarantee) + D (Midea as strategic customer
+partner). Triangulation 3/3 with verified anchor identity and
+voting power. C7 catalysts dated (Midea JV ramp H2 2026; cost-out
+H1 2027). No active red flags.
+This is the canonical Nordic Bucket A pattern that historically
+delivered 3-5x compounding (Wärtsilä, Atlas Copco split, SEB 2016
+rights). The Midea D-archetype layer is what makes the asymmetry
+meaningful — without the JV this would be a 2x normalisation
+trade; with it, the cycle + market-access combination supports
+base case 2.2x and bull 4.0x.
+Best Nordic recap candidate on the current screen.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="49">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Guaranty Trust Holding Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GTCO  ·  NG  ·  Bucket A  ·  Archetype G, A1  ·  Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.15×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.60× / 2.10× / 3.80×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>7.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.9×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>EM_bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>idiosyncratic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>G — Central Bank of Nigeria mandated capital floor of ₦500bn for international-licensed banks by 31 March 2026. GTCO recapped via ₦209bn local rights + ₦366bn LSE primary listing at ₦70 (2.28bn new shares). Total ₦575bn raised. Sector-wide CBN floor triggered ₦4.6tn in raises across all major Nigerian banks. CAR 15.20pct; Tier-1 capital +21pct YoY. Trades single-digit P/E + &lt;1x book despite &gt;20pct ROE due to Naira FX volatility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Naira stabilisation + FX policy normalisation</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.6-2.5× / Down -0.2--0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Sector consolidation — Nigerian smaller banks fail compliance</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.3-1.8× / Down -0.05--0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Pan-African expansion (UEMOA + East African subsidiaries)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2028-12-31</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.3-1.8× / Down -0.1--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Dividend re-rate (current yield distorted by Naira)</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-01 → 2028-12-31</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.2-1.5× / Down 0.0-0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: &lt;1x book at &gt;20pct ROE = &gt;25pct USD-adjusted earnings
+yield. Single-digit P/E.
+Leg 2: CBN-mandated capital floor = regulatory anchor;
+GTCO already over-complied; sector consolidation forces
+rivals to follow.
+Leg 3: LSE listing 2025 at ₦70 = revealed-preference floor
+by international institutional capital; UK pension fund
+interest demonstrates capital depth.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>GTCO retail + institutional float (LSE listing 2025), Pan-African pension + sovereign holders</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="n"/>
+      <c r="C41" s="19" t="n"/>
+      <c r="D41" s="19" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Naira FX volatility is the dominant variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="n"/>
+      <c r="C45" s="19" t="n"/>
+      <c r="D45" s="19" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Naira devalues another 30pct+ over 12 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>CBN-mandated forbearance escalates banking losses</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Heritage-Bank-style failure cascades across mid-tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Naira devalued to ₦3000/USD; GTCO USD-translated book and
+earnings collapsed; FX losses materialised; multiple
+contracted to 0.4x book.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n"/>
+      <c r="C53" s="19" t="n"/>
+      <c r="D53" s="19" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr"/>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype G (regulator-forced sector recap — canonical
+Yes Bank / Greek banks template) + A1 (LSE listing as sovereign-
+adjacent international float). Universe screen 0.79. Tier 1 on
+triangulation + dated regulatory floor + cleanest USD-adjusted
+asymmetric setup in MEA basket.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="37">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Hitachi Construction Machinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>6305  ·  JP  ·  Bucket A  ·  Archetype H, A1  ·  Tier 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>1.69×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.75× / 1.70× / 2.80×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>7.2×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.8×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Asian_governance_reform</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>H — Japan FIEA mandatory-TOB threshold cut from 33.3pct to 30pct effective May 1, 2026. Hitachi parent owns 30.7pct + Itochu 25pct = combined 55.7pct. Post-amendment Hitachi cannot rationally hold 30.7pct indefinitely: either step back below threshold or commit full TOB. Construction-machinery cycle inflection; HEC was carved out from Hitachi Construction Holdings 2007 - now a candidate parent-subsidiary buy-in (HEC-Itochu MBO precedent in 2022 Alps Logistics 194pct premium).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Hitachi parent decision on stake — step back below 30pct or full TOB</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-06-30</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.5-2.5× / Down -0.1--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Construction cycle inflection (mining + infrastructure + EV-mining)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2028-06-30</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.3-1.8× / Down -0.1--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Itochu strategic action (counter-bid or MBO partnership)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.6-2.2× / Down -0.05--0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: At 1.2x PBR not deeply undervalued vs sector; the
+alpha is in the takeout premium not the multiple gap.
+Leg 2: FIEA mandatory-TOB threshold has triggered for
+Hitachi parent. Game-theoretic option: step back (sale into
+market) or take out (TOB at premium). Either way creates
+forced flow.
+Leg 3: PARTIAL — Alps Logistics 194pct TOB premium (Itochu
+template) and Hitachi-Logisteed 40pct sale to KKR Apr 2023
+are precedents but no Hitachi statement of intent on HEC yet.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Hitachi Ltd parent (30.7pct), Itochu Corp (25.0pct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="n"/>
+      <c r="C44" s="19" t="n"/>
+      <c r="D44" s="19" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Japan FIEA enforcement grace period extended &gt;24 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Hitachi parent announces 'long-term hold' positioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Construction cycle deepens beyond 2026 trough</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Itochu strategically retreats from machinery sector</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is end-2027 and 6305 is down 50pct from current.
+Most likely: Hitachi parent given long FIEA enforcement
+grace period; no TOB; construction cycle weakened on global
+CapEx slowdown; multiple compressed.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n"/>
+      <c r="C53" s="19" t="n"/>
+      <c r="D53" s="19" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr"/>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype H (governance reset via FIEA forced
+decision) + A1 (parent + Itochu as combined 55.7pct cap-stack
+anchor). Universe screen 0.86. Tier 2 because catalyst is dated
+but binary on Hitachi parent's specific decision.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="38">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Drake &amp; Scull International</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DSI  ·  AE  ·  Bucket A  ·  Archetype E  ·  Tier 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.25×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.55× / 2.30× / 4.20×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>7.1×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.8×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>EM_bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>idiosyncratic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2024-04-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>E — UAE-equivalent restructuring with capital restoration. April 2024: AED 4.18bn debt write-off (90pct); AED 600m mandatory convertible sukuk issued; AED 800m capital reduction. Tabarak Investment (strategic since 2017) increased stake. Trading resumed May 2024 after 5-year halt. CEO Mansour Lootah leading recovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Backlog rebuild (UAE/GCC infrastructure pipeline)</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2028-06-30</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.8-2.5× / Down -0.2--0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Convertible sukuk conversion + capital structure simplification</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.3-1.6× / Down -0.1--0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Tabarak strategic-buyer follow-on or international JV partner</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2028-12-31</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.8-2.5× / Down -0.05--0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: Post-recap cap structure clean; 90pct of legacy debt
+written off creates large operating leverage to backlog
+rebuild. But absolute valuation tough without normalised
+EBITDA reference.
+Leg 2: Tabarak in since 2017 = patient anchor + UAE
+sovereign-adjacent capital base.
+Leg 3: AED 4.18bn debt forgiveness = creditor revealed
+preference for survival over liquidation.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Tabarak Investment (strategic anchor 2017+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>5-year trading halt history; legacy litigation overhang; limited float</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="n"/>
+      <c r="C44" s="19" t="n"/>
+      <c r="D44" s="19" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Second restructuring needed before 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Tabarak reduces stake</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Backlog material below normalised expectations through 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="n"/>
+      <c r="C49" s="19" t="n"/>
+      <c r="D49" s="19" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="20" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is end-2027 and DSI is down 60pct.
+Most likely: Backlog rebuild stalled; legacy litigation
+reactivated; GCC infrastructure cycle slowed; second
+restructuring or distressed equity raise.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="n"/>
+      <c r="C52" s="19" t="n"/>
+      <c r="D52" s="19" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype E (national bankruptcy framework / DIFC
+restructuring). Universe-screener 0.78 (15th). Tier 2 because
+legacy 5-year-halt history + low float + limited operational
+evidence post-recap. Builds for diversification within MEA
+basket; complements GTCO Nigerian recap basket exposure.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="37">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Doosan Bobcat (+ Doosan Robotics merger)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>241560  ·  KR  ·  Bucket A  ·  Archetype H, E  ·  Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>1.66×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.75× / 1.70× / 2.50×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>6.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.7×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Asian_governance_reform</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>H + E — Korean H6 governance overhaul. Aug 2024 original stock-swap proposal blocked by minority opposition + K-FSC ruling original ratio undervalued Bobcat. Q2 2026 revised terms tabled; Doosan Group cannot drop restructuring. Korean Commercial Act third amendment effective March 6, 2026 mandates treasury-share cancellation + cumulative voting for large companies + strengthened minority-shareholder rights — reform forcing chaebol governance overhaul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Revised stock-swap terms approved at Q2 2026 EGM (or alternative restructuring)</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2026-12-31</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.4-2.0× / Down -0.1--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Treasury-share cancellation announcement (Commercial Act compliance)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-09-01 → 2027-09-06</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.2-1.5× / Down -0.05--0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Korea Value-Up cohort re-rating (chaebol holdcos + treasury cancellation cascade)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2028-06-30</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.3-1.8× / Down -0.1--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: Bobcat at materially below SOTP; Robotics premium
+reflects valuation gap.
+Leg 2: Three forcing functions converge — Q2 2026 revised
+terms, Commercial Act amendment, treasury-share deadlines.
+Leg 3: K-FSC original-ratio rejection = revealed-preference
+floor; minority shareholders showed they can block; Park
+family must engage in good faith.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Doosan Group (Park family), Korea Value-Up framework + K-FSC enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="n"/>
+      <c r="C44" s="19" t="n"/>
+      <c r="D44" s="19" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Park family abandons restructuring; Bobcat trades as standalone</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Construction cycle deepens; Bobcat margins compress</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Doosan Group financial stress forces distressed disposal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="n"/>
+      <c r="C49" s="19" t="n"/>
+      <c r="D49" s="19" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="20" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is end-2027 and 241560 is down 50pct.
+Most likely: Restructuring postponed; chaebol family
+prioritised group-level liquidity needs; construction cycle
+weakened; multiple compressed.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="n"/>
+      <c r="C52" s="19" t="n"/>
+      <c r="D52" s="19" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype H (governance overhaul via K-FSC + Korean
+reform regime) + E (court/regulatory-sanctioned restructuring).
+Universe-screener 0.86. Tier 1 on multiple dated triggers
++ clear forcing functions + minority-shareholder protection
+precedent established.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="37">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Eutelsat Communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ETL  ·  FR  ·  Bucket A  ·  Archetype A1, F  ·  Tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Risk-reward snapshot</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Expected EV×</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.35×</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Bear / Base / Bull return</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>0.50× / 2.20× / 4.50×</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Bear loss</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Skew (upside/downside)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>7.0×</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Reward/Risk ratio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.7×</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Portfolio weight</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>French_sovereign</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Primary factor</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Mechanic</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Two-tier capital raise: c.€830m reserved increase to French State/Bharti/UK Gov/CMA CGM at premium price + €670m 8-for-11 rights at €1.35 (settled Dec 16, 2025); part of c.€1.5bn package with €4bn investment programme through 2026-2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>D2 Issue Discount Pct</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>D3 Backstop Cost Pct</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>D4 Dilution Pct</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>D5 Delta Wam Months</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>D6 Debt Tranches Post</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>D7 Ucc Terminations Pm30D</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>D8 Mip Strike Over Recap</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>D9 Alignment Gap</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>D9B Anchor Premium To Recap</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>D9C Premium To Vwap</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>D9D Liquidation Recovery Pct</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>D11 Consensus Ebitda Cagr</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>D13 Altman Z</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>D14 Liquidity Quarters</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Catalysts</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>P(yes)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Re-rate if yes / hit if no</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>IRIS² European sovereign LEO constellation operational milestones</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-01 → 2029-12-31</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.8-3.5× / Down -0.3--0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>OneWeb integration / commercial revenue synergies</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2027-12-31</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>Up 1.5-2.5× / Down -0.2--0.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Defence broadband contract wins (EU Strategic Compass)</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-01 → 2028-06-30</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Up 1.4-2.2× / Down -0.1--0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Triangulation (3-leg test)</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Leg 1 — Valuation</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Leg 2 — Game theory</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Leg 3 — Revealed preference</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leg 1: Pre-IRIS² EBITDA ~€800m on cap c.€2.5bn = EV/EBITDA ~3.5x PF
+vs SES 5-6x, Iridium 12x. Clear through-cycle asymmetry.
+Leg 2: Sovereign + strategic anchors with no fee/warrant kicker, no
+cramdown, no DIP. Lockup 6 months from settlement.
+Leg 3: The reserved capital increase TO ANCHORS at a premium price
+while parallel rights cleared at €1.35 is itself the revealed-
+preference signal. Current market €2.84 sits between anchor entry
+€4.00 and rights price €1.35, so partial re-rate priced.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Anchor</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="n"/>
+      <c r="C46" s="19" t="n"/>
+      <c r="D46" s="19" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>Parties</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>French State (APE), Bharti Space, UK Government, CMA CGM, FSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>Stake (% est.)</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Red flags</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>Triggered</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>None of 11 active</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>Watch list</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Kill criteria</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>IRIS² programme delay &gt;12 months announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Sovereign anchor exits lockup early or sells below cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>OneWeb integration write-down &gt;€500m</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>SES/Starlink pricing war causes &gt;20% revenue impairment</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Quarterly LEO connectivity revenue growth decelerates below 0% YoY</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Pre-mortem</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="n"/>
+      <c r="C61" s="19" t="n"/>
+      <c r="D61" s="19" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="20" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is end-2028 and ETL is down 70% from current ~€2.84.
+Most likely cause: IRIS² programme suffered material delays
+(mechanical: launch failures or contractor disputes; political:
+EU budget renegotiation under fiscal pressure). Eutelsat's role
+was reduced or contract terms re-cut. Concurrently, Starlink
+cleared regulatory hurdles for direct-to-cell competing with
+OneWeb in the same orbits, compressing OneWeb commercial value
+and triggering a goodwill write-down.
+Second-most-likely cause: SES merged with another operator and
+became a more aggressive competitor on price; LEO connectivity
+revenue growth decelerated; the partial re-rate from €1.35
+reversed back below €1.50.
+Where this would show up first: IRIS² programme milestone slips
+in EU Commission updates; Starlink direct-to-cell regulatory
+approvals; quarterly OneWeb revenue disclosure in interim reports.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Tier rationale</t>
+        </is>
+      </c>
+      <c r="B64" s="19" t="n"/>
+      <c r="C64" s="19" t="n"/>
+      <c r="D64" s="19" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bucket A, Archetype A1 (sovereign-strategic dual-tier raise) + F
+(post-recap orphan). Triangulation 3/3 with verified anchor
+presence. C7 partially visible (Q3 +3.1% YoY revenue, LEO-driven).
+IMPORTANT CORRECTION: The alignment gap is 1.41× not 2.9× as
+previously documented in shortlist.md. Current market €2.84 vs
+anchor €4.00 reserved. The €1.35 rights price is not the relevant
+denominator — the market price at announcement is. Lesson logged
+in methodology_review.md §1.4.
+Still investable but at narrower asymmetry than the prior screen
+implied. Remains Tier 1 on triangulation + C7 + dated catalyst
+basis but the "obvious mispricing" framing is weaker after the
+partial re-rate to €2.84 from late-Dec 2025 low ~€2.00.
+</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="49">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Regenerate deliverables over the expanded post-reorg universe
Listed-equity watchlist grows from 16 -> 56 tradable listed-common names
(41 filer-confirmed) after the 12x catch improvement flowed through: now
includes Diebold Nixdorf, SandRidge, Armstrong World, Tidewater, Par Pacific,
Visteon, Victoria's Secret, Sinclair, Gulfport, Bristow, Golar LNG, etc.
Broadsheet ledger + Excel workbook rebuilt to match.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVNbiVw8xFVKcK527PvUF9
</commit_message>
<xml_diff>
--- a/output/cyclepapa_risk_reward_workbook.xlsx
+++ b/output/cyclepapa_risk_reward_workbook.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -875,12 +875,12 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Valaris Ltd</t>
+          <t>DIEBOLD NIXDORF, Inc</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>VAL</t>
+          <t>DBD</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>August 12, 2023</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -930,19 +930,19 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>filer emerged 2021 (~61mo ago) — overhang likely cleared; low le</t>
+          <t>filer emerged August 12, 2023 (~35mo ago) — overhang likely clea</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>CBL &amp; ASSOCIATES PROPERTIES IN</t>
+          <t>Valaris Ltd</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>CBL</t>
+          <t>VAL</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -992,24 +992,24 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>net cash balance sheet; EBIT/EV 2% (neutral (0-20%))</t>
+          <t>filer emerged 2021 (~61mo ago) — overhang likely cleared; low le</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>California Resources Corp</t>
+          <t>CBL &amp; ASSOCIATES PROPERTIES IN</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>CBL</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
@@ -1054,29 +1054,29 @@
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 2.3×); EBIT/EV 13% (neutral (0-20%))</t>
+          <t>net cash balance sheet; EBIT/EV 2% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>RMR GROUP INC.</t>
+          <t>SANDRIDGE ENERGY INC</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>RMR</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>October 4, 2016</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -1116,29 +1116,29 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>net cash balance sheet; positive EBIT</t>
+          <t>filer emerged October 4, 2016 (~118mo ago) — overhang likely cle</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>APA Corp</t>
+          <t>ARMSTRONG WORLD INDUSTRIES INC</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AWI</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -1178,19 +1178,19 @@
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 25% (PRIORITY (&gt;20%))</t>
+          <t>filer emerged 2006 (~241mo ago) — overhang likely cleared; low l</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>WW INTERNATIONAL, INC.</t>
+          <t>TIDEWATER INC</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>TDW</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -1200,59 +1200,59 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>March 31, 2026</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>●</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>forced-creditor overhang</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>filer emerged March 31, 2026 (~4mo ago) — live forced-seller ove</t>
+          <t>filer emerged 2017 (~109mo ago) — overhang likely cleared; low l</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>WOLFSPEED, INC.</t>
+          <t>STIFEL FINANCIAL CORP</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>WOLF</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -1262,59 +1262,59 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>January 29, 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="G13" s="14" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>●</t>
         </is>
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>forced-creditor overhang</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="14" t="inlineStr">
         <is>
-          <t>filer emerged January 29, 2026 (~6mo ago) — live forced-seller o</t>
+          <t>net cash balance sheet; EBIT/EV 2% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Nine Energy Service, Inc.</t>
+          <t>ITRON, INC.</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>NINE</t>
+          <t>ITRI</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -1339,19 +1339,19 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
           <t>●</t>
@@ -1364,19 +1364,19 @@
       </c>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 0% (neutral (0-20%))</t>
+          <t>low leverage (ND/EBIT 0.7×); EBIT/EV 7% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Red Rock Resorts, Inc.</t>
+          <t>PAR PACIFIC HOLDINGS, INC.</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>PARR</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>August 31, 2012</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
@@ -1401,19 +1401,19 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I15" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
           <t>●</t>
@@ -1426,19 +1426,19 @@
       </c>
       <c r="L15" s="14" t="inlineStr">
         <is>
-          <t>filer emerged 2011 (~181mo ago) — overhang likely cleared; posit</t>
+          <t>filer emerged August 31, 2012 (~167mo ago) — overhang likely cle</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>SEADRILL Ltd</t>
+          <t>VISTEON CORP</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>SDRL</t>
+          <t>VC</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -1463,19 +1463,19 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="I16" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
           <t>●</t>
@@ -1488,19 +1488,19 @@
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 2% (neutral (0-20%))</t>
+          <t>net cash balance sheet; EBIT/EV 1% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Energy One, LLC</t>
+          <t>Spok Holdings, Inc</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>PHXE-P</t>
+          <t>SPOK</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -1525,19 +1525,19 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I17" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
           <t>●</t>
@@ -1550,19 +1550,19 @@
       </c>
       <c r="L17" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 4% (neutral (0-20%))</t>
+          <t>filer emerged 2002 (~289mo ago) — overhang likely cleared; net c</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Noble Corp plc</t>
+          <t>HOULIHAN LOKEY, INC.</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>HLI</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -1587,19 +1587,19 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
           <t>●</t>
@@ -1612,19 +1612,19 @@
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 5% (neutral (0-20%))</t>
+          <t>net cash balance sheet; positive EBIT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>NEXSTAR MEDIA GROUP, INC.</t>
+          <t>Victoria's Secret &amp; Co.</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>VSCO</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="I19" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I19" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
           <t>●</t>
@@ -1674,56 +1674,56 @@
       </c>
       <c r="L19" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 6% (neutral (0-20%))</t>
+          <t>filer emerged 2019 (~85mo ago) — overhang likely cleared; low le</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Capstone Energy Plus, Inc.</t>
+          <t>Diversified Energy Co</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>CGEH</t>
+          <t>DEC</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>July 4, 2025</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="I20" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
           <t>●</t>
@@ -1731,24 +1731,24 @@
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>forced-creditor overhang</t>
         </is>
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 1% (neutral (0-20%))</t>
+          <t>filer emerged July 4, 2025 (~13mo ago) — live forced-seller over</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>GoHealth, Inc.</t>
+          <t>Sinclair, Inc.</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>GOCO</t>
+          <t>SBGI</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
@@ -1773,86 +1773,2618 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="I21" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I21" s="14" t="inlineStr">
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L21" s="14" t="inlineStr">
+        <is>
+          <t>net cash balance sheet; positive EBIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Venture Global, Inc.</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J21" s="14" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K21" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L21" s="14" t="inlineStr"/>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>forced-creditor overhang</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>filer emerged 2025 (~13mo ago) — live forced-seller overhang; po</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>California Resources Corp</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L23" s="14" t="inlineStr">
+        <is>
+          <t>low leverage (ND/EBIT 2.3×); EBIT/EV 13% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Set aside — filer's own emergence unconfirmed (verify; not scored, not dropped)</t>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>INFINITY NATURAL RESOURCES, IN</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>low leverage (ND/EBIT 0.7×); positive EBIT</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Filing context</t>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Jefferies Financial Group Inc.</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>JEF</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>excess-emergence-cash</t>
+        </is>
+      </c>
+      <c r="L25" s="14" t="inlineStr">
+        <is>
+          <t>net cash balance sheet; net cash = 107% of mkt cap (net-debt bur</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>EASTMAN CHEMICAL CO</t>
+          <t>GULFPORT ENERGY CORP</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>EMN</t>
+          <t>GPOR</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>(bankruptcy reference is a non-filer possessive)</t>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="11" t="inlineStr">
+        <is>
+          <t>low leverage (ND/EBIT 1.3×); EBIT/EV 15% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
+          <t>AGCO CORP /DE</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>AGCO</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I27" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J27" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="14" t="inlineStr">
+        <is>
+          <t>low leverage (ND/EBIT 3.0×); EBIT/EV 4% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Bristow Group Inc.</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>VTOL</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="inlineStr">
+        <is>
+          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 7% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>RMR GROUP INC.</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>RMR</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I29" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J29" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K29" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L29" s="14" t="inlineStr">
+        <is>
+          <t>net cash balance sheet; positive EBIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>APA Corp</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K30" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L30" s="11" t="inlineStr">
+        <is>
+          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 25% (PRIORITY (&gt;20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>WW INTERNATIONAL, INC.</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>WW</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>December 31, 2025</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I31" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J31" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K31" s="14" t="inlineStr">
+        <is>
+          <t>forced-creditor overhang</t>
+        </is>
+      </c>
+      <c r="L31" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged December 31, 2025 (~7mo ago) — live forced-seller</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>WOLFSPEED, INC.</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>WOLF</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>January 29, 2026</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>forced-creditor overhang</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="inlineStr">
+        <is>
+          <t>filer emerged January 29, 2026 (~6mo ago) — live forced-seller o</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>GOLAR LNG LTD</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>GLNG</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I33" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="14" t="inlineStr">
+        <is>
+          <t>EBIT/EV 1% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Nine Energy Service, Inc.</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>NINE</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="inlineStr">
+        <is>
+          <t>EBIT/EV 0% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Red Rock Resorts, Inc.</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>RRR</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H35" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I35" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged 2011 (~181mo ago) — overhang likely cleared; posit</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>SEADRILL Ltd</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>SDRL</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="inlineStr">
+        <is>
+          <t>EBIT/EV 2% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Phoenix Energy One, LLC</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>PHXE-P</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H37" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I37" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J37" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K37" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" s="14" t="inlineStr">
+        <is>
+          <t>EBIT/EV 4% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Noble Corp plc</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K38" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" s="11" t="inlineStr">
+        <is>
+          <t>EBIT/EV 5% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>CLEVELAND-CLIFFS INC.</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>2042</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K39" s="14" t="inlineStr">
+        <is>
+          <t>forced-creditor overhang</t>
+        </is>
+      </c>
+      <c r="L39" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged 2042 (~-192mo ago) — live forced-seller overhang</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Capstone Green Energy Holdings</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>CGEH</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="11" t="inlineStr">
+        <is>
+          <t>EBIT/EV 1% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>NEXSTAR MEDIA GROUP, INC.</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>NXST</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I41" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J41" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K41" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="14" t="inlineStr">
+        <is>
+          <t>EBIT/EV 6% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>TruBridge, Inc.</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>TBRG</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="11" t="inlineStr">
+        <is>
+          <t>filer emerged 2020 (~73mo ago) — overhang likely cleared; EBIT/E</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Clean Energy Fuels Corp.</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>CLNE</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>September 1, 2025</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K43" s="14" t="inlineStr">
+        <is>
+          <t>forced-creditor overhang</t>
+        </is>
+      </c>
+      <c r="L43" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged September 1, 2025 (~11mo ago) — live forced-seller</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Smart Sand, Inc.</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>SND</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K44" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="11" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Sila Realty Trust, Inc.</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>SILA</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>February 16, 2024</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H45" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J45" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K45" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L45" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged February 16, 2024 (~29mo ago) — overhang likely cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>CLOVER HEALTH INVESTMENTS, COR</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>CLOV</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K46" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="11" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>Sable Offshore Corp.</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H47" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J47" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K47" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L47" s="14" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Ridgepost Capital, Inc.</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>RPC</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>May 3, 2017</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J48" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K48" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L48" s="11" t="inlineStr">
+        <is>
+          <t>filer emerged May 3, 2017 (~111mo ago) — overhang likely cleared</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>FERRELLGAS PARTNERS L P</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>FGPR</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G49" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H49" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J49" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K49" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" s="14" t="inlineStr">
+        <is>
+          <t>EBIT/EV 3% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>EchoStar CORP</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>SATS</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J50" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K50" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L50" s="11" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>Fortune Brands Innovations, In</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>FBIN</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G51" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H51" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J51" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K51" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L51" s="14" t="inlineStr">
+        <is>
+          <t>EBIT/EV 5% (neutral (0-20%))</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Beneficient</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>Fifth Era Acquisition Corp I</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>FERA</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H53" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J53" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K53" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L53" s="14" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>Xanadu Quantum Technologies Lt</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>XNDU</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J54" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K54" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L54" s="11" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>Cinemark Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>CNK</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>August 7, 2023</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H55" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I55" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J55" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K55" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L55" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged August 7, 2023 (~35mo ago) — overhang likely clear</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>iHeartMedia, Inc.</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>IHRT</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>May 1, 2019</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J56" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K56" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L56" s="11" t="inlineStr">
+        <is>
+          <t>filer emerged May 1, 2019 (~87mo ago) — overhang likely cleared</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>Tronox Holdings plc</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>TROX</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>November 30, 2010</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H57" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I57" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J57" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K57" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L57" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged November 30, 2010 (~188mo ago) — overhang likely c</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>GoHealth, Inc.</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>GOCO</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J58" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K58" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L58" s="11" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>Core Scientific, Inc./tx</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>CORZ</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H59" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I59" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J59" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K59" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L59" s="14" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Atlanta Braves Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>BATRA</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J60" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K60" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L60" s="11" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>AMPCO PITTSBURGH CORP</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="G61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K61" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L61" s="14" t="inlineStr"/>
+    </row>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Set aside — filer's own emergence unconfirmed (verify; not scored, not dropped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Filing context</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>OCTAVE SPECIALTY GROUP INC</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>OSG</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>EASTMAN CHEMICAL CO</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>EMN</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
           <t>PG&amp;E Corp</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B68" s="11" t="inlineStr">
         <is>
           <t>PCG</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>National CineMedia, Inc.</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>NCMI</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>MODIV INDUSTRIAL, INC.</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>MDV</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>LibreMax Asset-Backed Income F</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr"/>
+      <c r="C71" s="14" t="inlineStr">
         <is>
           <t>(bankruptcy reference is a non-filer possessive)</t>
         </is>

</xml_diff>

<commit_message>
Regenerate deliverables with Item 1.03 recoveries in the cohort
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVNbiVw8xFVKcK527PvUF9
</commit_message>
<xml_diff>
--- a/output/cyclepapa_risk_reward_workbook.xlsx
+++ b/output/cyclepapa_risk_reward_workbook.xlsx
@@ -617,7 +617,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Generated 2026-07-21</t>
+          <t>Generated 2026-07-22</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="M30" s="11" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 25% (PRIORITY (&gt;20%))</t>
+          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 24% (PRIORITY (&gt;20%))</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="M38" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 5% (neutral (0-20%))</t>
+          <t>EBIT/EV 4% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="M55" s="14" t="inlineStr">
         <is>
-          <t>filer emerged August 7, 2023 (~35mo ago) — overhang likely clear</t>
+          <t>filer emerged August 7, 2023 (~36mo ago) — overhang likely clear</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate deliverables: MCDIF + global post-reorgs captured, US ones fully scored
Listed-equity watchlist now spans 73 listed-common names incl. hand-curated
post-reorgs universe.md carried but the EDGAR poller couldn't: US filers
(Peabody, Warrior Met, Alpha Met) fully scored on SEC financials; OTC/foreign
(McDermott/MCDIF, Vallourec, Solocal, Orpea) captured with price+liquidity and
flagged. Ledger + workbook rebuilt.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVNbiVw8xFVKcK527PvUF9
</commit_message>
<xml_diff>
--- a/output/cyclepapa_risk_reward_workbook.xlsx
+++ b/output/cyclepapa_risk_reward_workbook.xlsx
@@ -709,11 +709,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -1958,17 +1958,17 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>California Resources Corp</t>
+          <t>Warrior Met Coal</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>NYSE:HCC</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
@@ -2018,19 +2018,19 @@
       </c>
       <c r="M23" s="14" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 2.3×); EBIT/EV 13% (neutral (0-20%))</t>
+          <t>net cash balance sheet; EBIT/EV 1% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>INFINITY NATURAL RESOURCES, IN</t>
+          <t>California Resources Corp</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -2085,19 +2085,19 @@
       </c>
       <c r="M24" s="11" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 0.7×); positive EBIT</t>
+          <t>low leverage (ND/EBIT 2.3×); EBIT/EV 13% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Jefferies Financial Group Inc.</t>
+          <t>INFINITY NATURAL RESOURCES, IN</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>JEF</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -2132,39 +2132,39 @@
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="J25" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
-          <t>excess-emergence-cash</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="14" t="inlineStr">
         <is>
-          <t>net cash balance sheet; net cash = 106% of mkt cap (net-debt bur</t>
+          <t>low leverage (ND/EBIT 0.7×); positive EBIT</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>GULFPORT ENERGY CORP</t>
+          <t>Jefferies Financial Group Inc.</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>GPOR</t>
+          <t>JEF</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -2199,39 +2199,39 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J26" s="11" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="L26" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>excess-emergence-cash</t>
         </is>
       </c>
       <c r="M26" s="11" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 1.3×); EBIT/EV 15% (neutral (0-20%))</t>
+          <t>net cash balance sheet; net cash = 106% of mkt cap (net-debt bur</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>AGCO CORP /DE</t>
+          <t>GULFPORT ENERGY CORP</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>AGCO</t>
+          <t>GPOR</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -2286,19 +2286,19 @@
       </c>
       <c r="M27" s="14" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 3.0×); EBIT/EV 4% (neutral (0-20%))</t>
+          <t>low leverage (ND/EBIT 1.3×); EBIT/EV 15% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Bristow Group Inc.</t>
+          <t>AGCO CORP /DE</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>VTOL</t>
+          <t>AGCO</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -2353,19 +2353,19 @@
       </c>
       <c r="M28" s="11" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 7% (neutral (0-20%))</t>
+          <t>low leverage (ND/EBIT 3.0×); EBIT/EV 4% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>RMR GROUP INC.</t>
+          <t>Bristow Group Inc.</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>RMR</t>
+          <t>VTOL</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr">
@@ -2420,19 +2420,19 @@
       </c>
       <c r="M29" s="14" t="inlineStr">
         <is>
-          <t>net cash balance sheet; positive EBIT</t>
+          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 7% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>APA Corp</t>
+          <t>RMR GROUP INC.</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>RMR</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -2487,86 +2487,86 @@
       </c>
       <c r="M30" s="11" t="inlineStr">
         <is>
-          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 24% (PRIORITY (&gt;20%))</t>
+          <t>net cash balance sheet; positive EBIT</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>WW INTERNATIONAL, INC.</t>
+          <t>APA Corp</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>~</t>
         </is>
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>December 31, 2025</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="H31" s="14" t="inlineStr">
+      <c r="I31" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I31" s="14" t="inlineStr">
+      <c r="J31" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J31" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>●</t>
         </is>
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>forced-creditor overhang</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="14" t="inlineStr">
         <is>
-          <t>filer emerged December 31, 2025 (~7mo ago) — live forced-seller</t>
+          <t>low leverage (ND/EBIT 2.7×); EBIT/EV 24% (PRIORITY (&gt;20%))</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>WOLFSPEED, INC.</t>
+          <t>WW INTERNATIONAL, INC.</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>WOLF</t>
+          <t>WW</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>January 29, 2026</t>
+          <t>December 31, 2025</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -2621,19 +2621,19 @@
       </c>
       <c r="M32" s="11" t="inlineStr">
         <is>
-          <t>filer emerged January 29, 2026 (~6mo ago) — live forced-seller o</t>
+          <t>filer emerged December 31, 2025 (~7mo ago) — live forced-seller</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>GOLAR LNG LTD</t>
+          <t>WOLFSPEED, INC.</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>GLNG</t>
+          <t>WOLF</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>January 29, 2026</t>
         </is>
       </c>
       <c r="E33" s="14" t="inlineStr">
@@ -2658,49 +2658,49 @@
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H33" s="14" t="inlineStr">
+      <c r="I33" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I33" s="14" t="inlineStr">
+      <c r="J33" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J33" s="14" t="inlineStr">
+      <c r="K33" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K33" s="14" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>forced-creditor overhang</t>
         </is>
       </c>
       <c r="M33" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 1% (neutral (0-20%))</t>
+          <t>filer emerged January 29, 2026 (~6mo ago) — live forced-seller o</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Nine Energy Service, Inc.</t>
+          <t>GOLAR LNG LTD</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>NINE</t>
+          <t>GLNG</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>thin</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="M34" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 0% (neutral (0-20%))</t>
+          <t>EBIT/EV 1% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>Red Rock Resorts, Inc.</t>
+          <t>Nine Energy Service, Inc.</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>NINE</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E35" s="14" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>thin</t>
         </is>
       </c>
       <c r="G35" s="14" t="inlineStr">
@@ -2822,19 +2822,19 @@
       </c>
       <c r="M35" s="14" t="inlineStr">
         <is>
-          <t>filer emerged 2011 (~181mo ago) — overhang likely cleared; posit</t>
+          <t>EBIT/EV 0% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>SEADRILL Ltd</t>
+          <t>Red Rock Resorts, Inc.</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>SDRL</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -2889,19 +2889,19 @@
       </c>
       <c r="M36" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 2% (neutral (0-20%))</t>
+          <t>filer emerged 2011 (~181mo ago) — overhang likely cleared; posit</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Energy One, LLC</t>
+          <t>SEADRILL Ltd</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>PHXE-P</t>
+          <t>SDRL</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>thin</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
@@ -2956,19 +2956,19 @@
       </c>
       <c r="M37" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 4% (neutral (0-20%))</t>
+          <t>EBIT/EV 2% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Noble Corp plc</t>
+          <t>Phoenix Energy One, LLC</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>PHXE-P</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>thin</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -3030,12 +3030,12 @@
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>CLEVELAND-CLIFFS INC.</t>
+          <t>Noble Corp plc</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>CLF</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>2042</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E39" s="14" t="inlineStr">
@@ -3060,49 +3060,49 @@
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J39" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K39" s="14" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="H39" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="I39" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="J39" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="K39" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L39" s="14" t="inlineStr">
         <is>
-          <t>forced-creditor overhang</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M39" s="14" t="inlineStr">
         <is>
-          <t>filer emerged 2042 (~-192mo ago) — live forced-seller overhang</t>
+          <t>EBIT/EV 4% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Capstone Green Energy Holdings</t>
+          <t>CLEVELAND-CLIFFS INC.</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>CGEH</t>
+          <t>CLF</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2042</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -3122,54 +3122,54 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H40" s="11" t="inlineStr">
+      <c r="I40" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I40" s="11" t="inlineStr">
+      <c r="J40" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J40" s="11" t="inlineStr">
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K40" s="11" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="L40" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>forced-creditor overhang</t>
         </is>
       </c>
       <c r="M40" s="11" t="inlineStr">
         <is>
-          <t>EBIT/EV 1% (neutral (0-20%))</t>
+          <t>filer emerged 2042 (~-192mo ago) — live forced-seller overhang</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>NEXSTAR MEDIA GROUP, INC.</t>
+          <t>Capstone Green Energy Holdings</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>CGEH</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G41" s="14" t="inlineStr">
@@ -3224,19 +3224,19 @@
       </c>
       <c r="M41" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 6% (neutral (0-20%))</t>
+          <t>EBIT/EV 1% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>TruBridge, Inc.</t>
+          <t>NEXSTAR MEDIA GROUP, INC.</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>TBRG</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -3291,19 +3291,19 @@
       </c>
       <c r="M42" s="11" t="inlineStr">
         <is>
-          <t>filer emerged 2020 (~73mo ago) — overhang likely cleared; EBIT/E</t>
+          <t>EBIT/EV 6% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>Clean Energy Fuels Corp.</t>
+          <t>TruBridge, Inc.</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>CLNE</t>
+          <t>TBRG</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>September 1, 2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="E43" s="14" t="inlineStr">
@@ -3323,54 +3323,54 @@
       </c>
       <c r="F43" s="14" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J43" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K43" s="14" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="H43" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="I43" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="J43" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="K43" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L43" s="14" t="inlineStr">
         <is>
-          <t>forced-creditor overhang</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M43" s="14" t="inlineStr">
         <is>
-          <t>filer emerged September 1, 2025 (~11mo ago) — live forced-seller</t>
+          <t>filer emerged 2020 (~73mo ago) — overhang likely cleared; EBIT/E</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>Smart Sand, Inc.</t>
+          <t>Clean Energy Fuels Corp.</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>SND</t>
+          <t>CLNE</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>September 1, 2025</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -3395,14 +3395,14 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H44" s="11" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
           <t>·</t>
@@ -3420,24 +3420,24 @@
       </c>
       <c r="L44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>forced-creditor overhang</t>
         </is>
       </c>
       <c r="M44" s="11" t="inlineStr">
         <is>
-          <t>net cash balance sheet</t>
+          <t>filer emerged September 1, 2025 (~11mo ago) — live forced-seller</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>Sila Realty Trust, Inc.</t>
+          <t>Smart Sand, Inc.</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>SILA</t>
+          <t>SND</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>February 16, 2024</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E45" s="14" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G45" s="14" t="inlineStr">
@@ -3467,24 +3467,24 @@
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I45" s="14" t="inlineStr">
+      <c r="J45" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J45" s="14" t="inlineStr">
+      <c r="K45" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K45" s="14" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="L45" s="14" t="inlineStr">
         <is>
           <t>—</t>
@@ -3492,19 +3492,19 @@
       </c>
       <c r="M45" s="14" t="inlineStr">
         <is>
-          <t>filer emerged February 16, 2024 (~29mo ago) — overhang likely cl</t>
+          <t>net cash balance sheet</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>CLOVER HEALTH INVESTMENTS, COR</t>
+          <t>Sila Realty Trust, Inc.</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>SILA</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>February 16, 2024</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -3534,24 +3534,24 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K46" s="11" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="I46" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="J46" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="K46" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L46" s="11" t="inlineStr">
         <is>
           <t>—</t>
@@ -3559,19 +3559,19 @@
       </c>
       <c r="M46" s="11" t="inlineStr">
         <is>
-          <t>net cash balance sheet</t>
+          <t>filer emerged February 16, 2024 (~29mo ago) — overhang likely cl</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>Sable Offshore Corp.</t>
+          <t>CLOVER HEALTH INVESTMENTS, COR</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>SOC</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">
@@ -3633,12 +3633,12 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>Ridgepost Capital, Inc.</t>
+          <t>Sable Offshore Corp.</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>SOC</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>May 3, 2017</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G48" s="11" t="inlineStr">
@@ -3668,24 +3668,24 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I48" s="11" t="inlineStr">
+      <c r="J48" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J48" s="11" t="inlineStr">
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K48" s="11" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="L48" s="11" t="inlineStr">
         <is>
           <t>—</t>
@@ -3693,29 +3693,29 @@
       </c>
       <c r="M48" s="11" t="inlineStr">
         <is>
-          <t>filer emerged May 3, 2017 (~111mo ago) — overhang likely cleared</t>
+          <t>net cash balance sheet</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>FERRELLGAS PARTNERS L P</t>
+          <t>Ridgepost Capital, Inc.</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>FGPR</t>
+          <t>RPC</t>
         </is>
       </c>
       <c r="C49" s="14" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>May 3, 2017</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="F49" s="14" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="G49" s="14" t="inlineStr">
@@ -3760,24 +3760,24 @@
       </c>
       <c r="M49" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 3% (neutral (0-20%))</t>
+          <t>filer emerged May 3, 2017 (~111mo ago) — overhang likely cleared</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>EchoStar CORP</t>
+          <t>Core Natural Resources</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>SATS</t>
+          <t>NYSE:CNR</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3834,17 +3834,17 @@
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>Fortune Brands Innovations, In</t>
+          <t>Alpha Metallurgical Resources</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>FBIN</t>
+          <t>NYSE:AMR</t>
         </is>
       </c>
       <c r="C51" s="14" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D51" s="14" t="inlineStr">
@@ -3869,24 +3869,24 @@
       </c>
       <c r="H51" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I51" s="14" t="inlineStr">
+      <c r="J51" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J51" s="14" t="inlineStr">
+      <c r="K51" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K51" s="14" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="L51" s="14" t="inlineStr">
         <is>
           <t>—</t>
@@ -3894,24 +3894,24 @@
       </c>
       <c r="M51" s="14" t="inlineStr">
         <is>
-          <t>EBIT/EV 5% (neutral (0-20%))</t>
+          <t>net cash balance sheet</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>Beneficient</t>
+          <t>Peabody Energy</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>BENF</t>
+          <t>NYSE:BTU</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr">
@@ -3968,12 +3968,12 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>Fifth Era Acquisition Corp I</t>
+          <t>FERRELLGAS PARTNERS L P</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>FERA</t>
+          <t>FGPR</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="F53" s="14" t="inlineStr">
         <is>
-          <t>thin</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="G53" s="14" t="inlineStr">
@@ -4003,24 +4003,24 @@
       </c>
       <c r="H53" s="14" t="inlineStr">
         <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J53" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K53" s="14" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="I53" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="J53" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="K53" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L53" s="14" t="inlineStr">
         <is>
           <t>—</t>
@@ -4028,19 +4028,19 @@
       </c>
       <c r="M53" s="14" t="inlineStr">
         <is>
-          <t>net cash balance sheet</t>
+          <t>EBIT/EV 3% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>Xanadu Quantum Technologies Lt</t>
+          <t>EchoStar CORP</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>XNDU</t>
+          <t>SATS</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
@@ -4102,27 +4102,27 @@
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>Cinemark Holdings, Inc.</t>
+          <t>Fortune Brands Innovations, In</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>CNK</t>
+          <t>FBIN</t>
         </is>
       </c>
       <c r="C55" s="14" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>~</t>
         </is>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>August 7, 2023</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F55" s="14" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="K55" s="14" t="inlineStr">
         <is>
-          <t>·</t>
+          <t>●</t>
         </is>
       </c>
       <c r="L55" s="14" t="inlineStr">
@@ -4162,39 +4162,39 @@
       </c>
       <c r="M55" s="14" t="inlineStr">
         <is>
-          <t>filer emerged August 7, 2023 (~36mo ago) — overhang likely clear</t>
+          <t>EBIT/EV 5% (neutral (0-20%))</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>iHeartMedia, Inc.</t>
+          <t>Beneficient</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>IHRT</t>
+          <t>BENF</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>~</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>May 1, 2019</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="G56" s="11" t="inlineStr">
@@ -4204,24 +4204,24 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I56" s="11" t="inlineStr">
+      <c r="J56" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J56" s="11" t="inlineStr">
+      <c r="K56" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K56" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
           <t>—</t>
@@ -4229,39 +4229,39 @@
       </c>
       <c r="M56" s="11" t="inlineStr">
         <is>
-          <t>filer emerged May 1, 2019 (~87mo ago) — overhang likely cleared</t>
+          <t>net cash balance sheet</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>Tronox Holdings plc</t>
+          <t>Fifth Era Acquisition Corp I</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>TROX</t>
+          <t>FERA</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>~</t>
         </is>
       </c>
       <c r="D57" s="14" t="inlineStr">
         <is>
-          <t>November 30, 2010</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E57" s="14" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>deep</t>
+          <t>thin</t>
         </is>
       </c>
       <c r="G57" s="14" t="inlineStr">
@@ -4271,24 +4271,24 @@
       </c>
       <c r="H57" s="14" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I57" s="14" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I57" s="14" t="inlineStr">
+      <c r="J57" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J57" s="14" t="inlineStr">
+      <c r="K57" s="14" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K57" s="14" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L57" s="14" t="inlineStr">
         <is>
           <t>—</t>
@@ -4296,24 +4296,24 @@
       </c>
       <c r="M57" s="14" t="inlineStr">
         <is>
-          <t>filer emerged November 30, 2010 (~188mo ago) — overhang likely c</t>
+          <t>net cash balance sheet</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>GoHealth, Inc.</t>
+          <t>Xanadu Quantum Technologies Lt</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>GOCO</t>
+          <t>XNDU</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>~</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4323,12 +4323,12 @@
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>deep</t>
         </is>
       </c>
       <c r="G58" s="11" t="inlineStr">
@@ -4338,40 +4338,44 @@
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I58" s="11" t="inlineStr">
+      <c r="J58" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J58" s="11" t="inlineStr">
+      <c r="K58" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K58" s="11" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M58" s="11" t="inlineStr"/>
+      <c r="M58" s="11" t="inlineStr">
+        <is>
+          <t>net cash balance sheet</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>Core Scientific, Inc./tx</t>
+          <t>Cinemark Holdings, Inc.</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>CORZ</t>
+          <t>CNK</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -4381,7 +4385,7 @@
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>August 7, 2023</t>
         </is>
       </c>
       <c r="E59" s="14" t="inlineStr">
@@ -4424,17 +4428,21 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M59" s="14" t="inlineStr"/>
+      <c r="M59" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged August 7, 2023 (~36mo ago) — overhang likely clear</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>Atlanta Braves Holdings, Inc.</t>
+          <t>iHeartMedia, Inc.</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>BATRA</t>
+          <t>IHRT</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
@@ -4444,7 +4452,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>May 1, 2019</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -4487,27 +4495,31 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M60" s="11" t="inlineStr"/>
+      <c r="M60" s="11" t="inlineStr">
+        <is>
+          <t>filer emerged May 1, 2019 (~87mo ago) — overhang likely cleared</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>AMPCO PITTSBURGH CORP</t>
+          <t>Tronox Holdings plc</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>TROX</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>November 30, 2010</t>
         </is>
       </c>
       <c r="E61" s="14" t="inlineStr">
@@ -4517,160 +4529,1283 @@
       </c>
       <c r="F61" s="14" t="inlineStr">
         <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K61" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L61" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M61" s="14" t="inlineStr">
+        <is>
+          <t>filer emerged November 30, 2010 (~188mo ago) — overhang likely c</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>GoHealth, Inc.</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>GOCO</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>micro</t>
+        </is>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J62" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K62" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L62" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M62" s="11" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>Core Scientific, Inc./tx</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>CORZ</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="inlineStr">
+        <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G63" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H63" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I63" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J63" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K63" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L63" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M63" s="14" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>Atlanta Braves Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>BATRA</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="G61" s="14" t="inlineStr">
+      <c r="G64" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="H61" s="14" t="inlineStr">
+      <c r="H64" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I61" s="14" t="inlineStr">
+      <c r="I64" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J61" s="14" t="inlineStr">
+      <c r="J64" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="K61" s="14" t="inlineStr">
+      <c r="K64" s="11" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="L61" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M61" s="14" t="inlineStr"/>
-    </row>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>Set aside — filer's own emergence unconfirmed (verify; not scored, not dropped)</t>
-        </is>
-      </c>
+      <c r="L64" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>Filing context</t>
-        </is>
-      </c>
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>PAL Holdings (Philippine Airli</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>PSE:PAL</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G65" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H65" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I65" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J65" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K65" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L65" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M65" s="14" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>OCTAVE SPECIALTY GROUP INC</t>
+          <t>AMPCO PITTSBURGH CORP</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>(bankruptcy reference is a non-filer possessive)</t>
-        </is>
-      </c>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G66" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I66" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J66" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K66" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L66" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t>EASTMAN CHEMICAL CO</t>
+          <t>McDermott International</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>EMN</t>
+          <t>OTC:MCDIF</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
         <is>
-          <t>(bankruptcy reference is a non-filer possessive)</t>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="inlineStr">
+        <is>
+          <t>thin</t>
+        </is>
+      </c>
+      <c r="G67" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H67" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I67" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J67" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K67" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L67" s="14" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M67" s="14" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>PG&amp;E Corp</t>
+          <t>Orpea / Emeis</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>PCG</t>
+          <t>EPA:EMEIS</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>(bankruptcy reference is a non-filer possessive)</t>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G68" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H68" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I68" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J68" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K68" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L68" s="11" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M68" s="11" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t>National CineMedia, Inc.</t>
+          <t>Vallourec</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>NCMI</t>
+          <t>EPA:VK</t>
         </is>
       </c>
       <c r="C69" s="14" t="inlineStr">
         <is>
-          <t>(bankruptcy reference is a non-filer possessive)</t>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="inlineStr">
+        <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G69" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H69" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I69" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J69" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K69" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L69" s="14" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M69" s="14" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>MODIV INDUSTRIAL, INC.</t>
+          <t>Solocal Group</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>MDV</t>
+          <t>EPA:LOCAL</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>(bankruptcy reference is a non-filer possessive)</t>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>micro</t>
+        </is>
+      </c>
+      <c r="G70" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H70" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I70" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J70" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K70" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L70" s="11" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M70" s="11" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
+          <t>Intrum</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>ST:INTRUM</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="inlineStr">
+        <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G71" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H71" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I71" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J71" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K71" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L71" s="14" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M71" s="14" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>Norwegian Air Shuttle</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>OSL:NAS</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G72" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H72" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I72" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J72" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K72" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L72" s="11" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M72" s="11" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>HMM (Hyundai Merchant Marine)</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>KRX:011200</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F73" s="14" t="inlineStr">
+        <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G73" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H73" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I73" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J73" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K73" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L73" s="14" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M73" s="14" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>Sri Rejeki Isman (Sritex)</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>IDX:SRIL</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H74" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I74" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J74" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K74" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L74" s="11" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M74" s="11" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>AirAsia X</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>KLSE:5238</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F75" s="14" t="inlineStr">
+        <is>
+          <t>deep</t>
+        </is>
+      </c>
+      <c r="G75" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H75" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J75" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K75" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L75" s="14" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M75" s="14" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>Lupatech</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>B3:LUPA3</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>micro</t>
+        </is>
+      </c>
+      <c r="G76" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H76" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K76" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L76" s="11" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M76" s="11" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>Drake &amp; Scull</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>DFM:DSI</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H77" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I77" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J77" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K77" s="14" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L77" s="14" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M77" s="14" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>OI SA</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>B3:OIBR3</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>micro</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="H78" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="J78" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="K78" s="11" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="L78" s="11" t="inlineStr">
+        <is>
+          <t>hand-curated post-reorg</t>
+        </is>
+      </c>
+      <c r="M78" s="11" t="inlineStr">
+        <is>
+          <t>universe.md Bucket C (OTC/foreign; SEC financials unavailable —</t>
+        </is>
+      </c>
+    </row>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>Set aside — filer's own emergence unconfirmed (verify; not scored, not dropped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Filing context</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>OCTAVE SPECIALTY GROUP INC</t>
+        </is>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>OSG</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>EASTMAN CHEMICAL CO</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>EMN</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>PG&amp;E Corp</t>
+        </is>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>PCG</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>National CineMedia, Inc.</t>
+        </is>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>NCMI</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>MODIV INDUSTRIAL, INC.</t>
+        </is>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>MDV</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>(bankruptcy reference is a non-filer possessive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
           <t>LibreMax Asset-Backed Income F</t>
         </is>
       </c>
-      <c r="B71" s="14" t="inlineStr"/>
-      <c r="C71" s="14" t="inlineStr">
+      <c r="B88" s="14" t="inlineStr"/>
+      <c r="C88" s="14" t="inlineStr">
         <is>
           <t>(bankruptcy reference is a non-filer possessive)</t>
         </is>

</xml_diff>